<commit_message>
fix(linx): validate v0.58 irregular tile operations
</commit_message>
<xml_diff>
--- a/docs/linxisa/qemu_tile_profile_support.xlsx
+++ b/docs/linxisa/qemu_tile_profile_support.xlsx
@@ -170,7 +170,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -265,17 +265,17 @@
         <v>248</v>
       </c>
       <c r="C9" s="3">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D9" s="4">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E9" s="5">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>11.3%</t>
+          <t>12.1%</t>
         </is>
       </c>
     </row>
@@ -286,20 +286,20 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C10" s="3">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D10" s="4">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E10" s="5">
         <v>1</v>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>16.3%</t>
         </is>
       </c>
     </row>
@@ -334,20 +334,20 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="C12" s="3">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="D12" s="4">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="E12" s="5">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>42.7%</t>
+          <t>43.4%</t>
         </is>
       </c>
     </row>
@@ -606,7 +606,7 @@
       </c>
       <c r="V2" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -719,7 +719,7 @@
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -832,7 +832,7 @@
       </c>
       <c r="V4" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -945,7 +945,7 @@
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="V6" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -1284,7 +1284,7 @@
       </c>
       <c r="V8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1621,7 @@
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -1734,7 +1734,7 @@
       </c>
       <c r="V12" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="V13" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -1960,7 +1960,7 @@
       </c>
       <c r="V14" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -2073,7 +2073,7 @@
       </c>
       <c r="V15" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       </c>
       <c r="V16" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -2299,7 +2299,7 @@
       </c>
       <c r="V17" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -2412,7 +2412,7 @@
       </c>
       <c r="V18" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -2525,7 +2525,7 @@
       </c>
       <c r="V19" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -2638,7 +2638,7 @@
       </c>
       <c r="V20" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="V21" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
       </c>
       <c r="V22" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="V23" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -3090,7 +3090,7 @@
       </c>
       <c r="V24" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -3427,7 +3427,7 @@
       </c>
       <c r="V27" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -3540,7 +3540,7 @@
       </c>
       <c r="V28" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -3653,7 +3653,7 @@
       </c>
       <c r="V29" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -3766,7 +3766,7 @@
       </c>
       <c r="V30" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -3879,7 +3879,7 @@
       </c>
       <c r="V31" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -3992,7 +3992,7 @@
       </c>
       <c r="V32" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -4105,7 +4105,7 @@
       </c>
       <c r="V33" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -4218,7 +4218,7 @@
       </c>
       <c r="V34" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -4331,7 +4331,7 @@
       </c>
       <c r="V35" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -4444,7 +4444,7 @@
       </c>
       <c r="V36" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -4879,7 +4879,7 @@
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -5456,7 +5456,7 @@
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -6993,7 +6993,7 @@
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -7186,7 +7186,7 @@
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -7379,7 +7379,7 @@
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -7572,7 +7572,7 @@
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -8208,9 +8208,9 @@
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M20" s="6" t="inlineStr">
@@ -8335,12 +8335,13 @@
       </c>
       <c r="AK20" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>v058_irregular_layout_profiles
+Automated current-ISA profile verification; evidence refs: textract_fp32.</t>
         </is>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -8769,121 +8770,121 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I23" s="5" t="inlineStr">
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="T23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="X23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Y23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Z23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AA23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AB23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AC23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AD23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AE23" s="5" t="inlineStr">
         <is>
           <t>UNSUPPORTED</t>
         </is>
       </c>
-      <c r="J23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="O23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="P23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Q23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="R23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="S23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="V23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Y23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Z23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AA23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AB23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AC23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AD23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AE23" s="5" t="inlineStr">
-        <is>
-          <t>UNSUPPORTED</t>
-        </is>
-      </c>
       <c r="AF23" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -8911,13 +8912,13 @@
       </c>
       <c r="AK23" s="7" t="inlineStr">
         <is>
-          <t>QEMU fail-closed support audit
-The current QEMU head rejects this identity/profile before destination mutation.</t>
+          <t>v058_irregular_layout_profiles
+Automated current-ISA profile verification; evidence refs: thistogram_u32_byte3.</t>
         </is>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -11418,7 +11419,7 @@
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -12955,7 +12956,7 @@
       </c>
       <c r="AL44" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -13148,7 +13149,7 @@
       </c>
       <c r="AL45" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -13341,7 +13342,7 @@
       </c>
       <c r="AL46" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -13534,7 +13535,7 @@
       </c>
       <c r="AL47" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -14687,7 +14688,7 @@
       </c>
       <c r="AL53" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -14736,8 +14737,9 @@
     <col min="33" max="33" width="14" customWidth="1"/>
     <col min="34" max="34" width="14" customWidth="1"/>
     <col min="35" max="35" width="14" customWidth="1"/>
-    <col min="36" max="36" width="58" customWidth="1"/>
-    <col min="37" max="37" width="14" customWidth="1"/>
+    <col min="36" max="36" width="14" customWidth="1"/>
+    <col min="37" max="37" width="58" customWidth="1"/>
+    <col min="38" max="38" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -14803,125 +14805,130 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Local FP16; valid 4x16; NORM row-major; PE-local 128B</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Local FP32; 16x16; NORM row-major; PE-local 1KiB</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Local FP32; 16x32; NORM row-major; PE-local 2KiB</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Local FP32; 32x32; NORM row-major; PE-local 4KiB</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Local FP32; 8x16; NORM row-major; PE-local 512B</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Local FP32; 8x32; NORM row-major; PE-local 1KiB</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Local NORM S8/U8/S16/U16/S32/U32/F32; logical row stride; valid rectangle</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Local S32; valid 4x8; NORM row-major; PE-local 128B</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>PTO TLOAD dtype/layout combinations supported by the v5 TLSU profile</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>PTO TSTORE dtype/layout combinations supported by the v5 TLSU profile</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Same element dtype set as TLOAD profile; src/dst element size must match</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Shared full FP32; PE0 issuer; K16xN32 NORM; PE-local 2KiB class 5; Core4 aggregate 8KiB</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Shared full FP32; PE0 issuer; K32xN16 NORM; PE-local 2KiB class 5; Core4 aggregate 8KiB</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Shared full FP32; PE0 issuer; K32xN32 NORM; PE-local 4KiB class 6; Core4 aggregate 16KiB</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Shared full S8; PE0 issuer; K16xN32 NORM; PE-local 512B class 3; Core4 aggregate 2KiB</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Shared full/core FP32; B.IOS source; Function 1; NORM</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Shared pe_scope FP32; B.IOS source; Function 14; NORM</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>TLSU atomic data types accepted by BSTART.MGATHER.CAS</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>TLSU data types accepted by BSTART.MGATHER.MASK</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>TLSU data types accepted by BSTART.MSCATTER.MASK</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>byte-preserving; descriptors must be compatible</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>byte-preserving; source and destination descriptors must match</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>data: S8</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>data: U8</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>Evidence / Notes</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>Last checked</t>
         </is>
@@ -15088,28 +15095,33 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AG2" s="5" t="inlineStr">
+      <c r="AG2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AH2" s="5" t="inlineStr">
         <is>
           <t>UNSUPPORTED</t>
         </is>
       </c>
-      <c r="AH2" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="AI2" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="AJ2" s="7" t="inlineStr">
+      <c r="AJ2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AK2" s="7" t="inlineStr">
         <is>
           <t>QEMU fail-closed support audit
 The current QEMU head rejects this identity/profile before destination mutation.</t>
         </is>
       </c>
-      <c r="AK2" s="7" t="inlineStr">
+      <c r="AL2" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -15156,9 +15168,9 @@
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -15286,19 +15298,25 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AI3" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="AJ3" s="7" t="inlineStr">
-        <is>
-          <t>MGATHER dst B.DATR PadValue.Null accepted per B.DATR.md PadValue table; index dtype gate enforces S32/U32 per MGATHER.md and fails closed before memory side effects. 91-case rerun: mgather_i32 PASS; mgather_fp16/fp32 and gelu_bf16 FAIL_ILLEGAL because their dst B.DATR DataType=31 is invalid (B.DATR.md), an ELF-side defect. Cell stays UNVERIFIED without an independent golden.</t>
+      <c r="AI3" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AJ3" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="AK3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>v058_irregular_layout_profiles
+Automated current-ISA profile verification; evidence refs: mgather_u32.</t>
+        </is>
+      </c>
+      <c r="AL3" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -15443,14 +15461,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AC4" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="AD4" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AC4" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AD4" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="AE4" s="6" t="inlineStr">
@@ -15478,12 +15496,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AJ4" s="7" t="inlineStr">
+      <c r="AJ4" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AK4" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="AK4" s="7" t="inlineStr">
+      <c r="AL4" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -15635,14 +15658,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AD5" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="AE5" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AD5" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AE5" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="AF5" s="6" t="inlineStr">
@@ -15665,12 +15688,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AJ5" s="7" t="inlineStr">
+      <c r="AJ5" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AK5" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="AK5" s="7" t="inlineStr">
+      <c r="AL5" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -15842,22 +15870,27 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AH6" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="AI6" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AJ6" s="7" t="inlineStr">
+      <c r="AH6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AI6" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="AJ6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AK6" s="7" t="inlineStr">
         <is>
           <t>Source-only stores accept TSize=000 and derive size from the source descriptor per B.IOT.md; index dtype gate enforces S32/U32 per MSCATTER.md and fails closed before memory side effects. 91-case rerun: mscatter_i32 PASS; mscatter_fp16/fp32 FAIL_ILLEGAL because their index tile dtype is FP16/FP32. Cell stays UNVERIFIED without an independent golden.</t>
         </is>
       </c>
-      <c r="AK6" s="7" t="inlineStr">
+      <c r="AL6" s="7" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
@@ -16014,14 +16047,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AE7" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="AF7" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AE7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AF7" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="AG7" s="6" t="inlineStr">
@@ -16039,12 +16072,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AJ7" s="7" t="inlineStr">
+      <c r="AJ7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AK7" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="AK7" s="7" t="inlineStr">
+      <c r="AL7" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -16111,34 +16149,34 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="M8" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="N8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="O8" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="P8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Q8" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="R8" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="O8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="S8" s="3" t="inlineStr">
@@ -16146,14 +16184,14 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="T8" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="U8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="U8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="V8" s="6" t="inlineStr">
@@ -16161,9 +16199,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="W8" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="W8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="X8" s="4" t="inlineStr">
@@ -16181,9 +16219,9 @@
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="AA8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AA8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="AB8" s="6" t="inlineStr">
@@ -16226,15 +16264,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AJ8" s="7" t="inlineStr">
-        <is>
-          <t>v058_tload_tile_state; v058_tload_tstore_common_profiles
-Automated current-ISA profile verification; evidence refs: fp32_row0, fp32_row1, s16_row0, s16_row1, s8_row0, s8_row1, u8_row0, u8_row1, u16_row0, u16_row1, s32_row0, s32_row1, u32_row0, u32_row1, zero_stride_rows.</t>
+      <c r="AJ8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AK8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>v058_tload_fp16_tile_state; v058_tload_tile_state; v058_tload_tstore_common_profiles
+Automated current-ISA profile verification; evidence refs: T#1.</t>
+        </is>
+      </c>
+      <c r="AL8" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -16394,14 +16437,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AF9" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="AG9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AF9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AG9" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="AH9" s="6" t="inlineStr">
@@ -16414,13 +16457,18 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AJ9" s="7" t="inlineStr">
+      <c r="AJ9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AK9" s="7" t="inlineStr">
         <is>
           <t>bin-20260806 matmul_MASK_MASK_FP32_REUSEA/B (full 356 rerun); TMOV.md byte-preserving descriptor inheritance fix
 TMOV materialize now inherits the bound source Tile shape for aliased (src==dst) moves; REUSEA/B FP32 flipped FAIL_ILLEGAL -&gt; PASS. Local TMOV with B.IOT dst is legal per TMOV.md; Shared modes (L2S Function 9-12) remain UNVERIFIED here.</t>
         </is>
       </c>
-      <c r="AK9" s="7" t="inlineStr">
+      <c r="AL9" s="7" t="inlineStr">
         <is>
           <t>2026-08-08</t>
         </is>
@@ -16532,14 +16580,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="V10" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="W10" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="V10" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W10" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="X10" s="6" t="inlineStr">
@@ -16602,12 +16650,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AJ10" s="7" t="inlineStr">
+      <c r="AJ10" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AK10" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="AK10" s="7" t="inlineStr">
+      <c r="AL10" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -16679,9 +16732,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="N11" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="N11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
@@ -16694,34 +16747,34 @@
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="Q11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="R11" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="S11" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="T11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U11" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="V11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="Q11" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="R11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T11" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="U11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V11" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="W11" s="6" t="inlineStr">
@@ -16744,9 +16797,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AA11" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="AA11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AB11" s="3" t="inlineStr">
@@ -16754,9 +16807,9 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="AC11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AC11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AD11" s="6" t="inlineStr">
@@ -16789,20 +16842,25 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AJ11" s="7" t="inlineStr">
+      <c r="AJ11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AK11" s="7" t="inlineStr">
         <is>
           <t>v058_shared_tlsu; v058_tload_tstore_common_profiles
 Automated current-ISA profile verification; evidence refs: fp32_row0, fp32_row1, s16_row0, s16_row1, s8_row0, s8_row1, u8_row0, u8_row1, u16_row0, u16_row1, s32_row0, s32_row1, u32_row0, u32_row1, zero_stride_rows.</t>
         </is>
       </c>
-      <c r="AK11" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="AL11" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AK11"/>
+  <autoFilter ref="A1:AL11"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>
@@ -17012,7 +17070,7 @@
       </c>
       <c r="R2" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -17105,7 +17163,7 @@
       </c>
       <c r="R3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -17198,7 +17256,7 @@
       </c>
       <c r="R4" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -17291,7 +17349,7 @@
       </c>
       <c r="R5" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -17384,7 +17442,7 @@
       </c>
       <c r="R6" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -17477,7 +17535,7 @@
       </c>
       <c r="R7" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -17570,7 +17628,7 @@
       </c>
       <c r="R8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -17663,7 +17721,7 @@
       </c>
       <c r="R9" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -17756,7 +17814,7 @@
       </c>
       <c r="R10" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -17849,7 +17907,7 @@
       </c>
       <c r="R11" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -17942,7 +18000,7 @@
       </c>
       <c r="R12" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -18035,7 +18093,7 @@
       </c>
       <c r="R13" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(tile): align PTO v0.58 compare and select semantics
</commit_message>
<xml_diff>
--- a/docs/linxisa/qemu_tile_profile_support.xlsx
+++ b/docs/linxisa/qemu_tile_profile_support.xlsx
@@ -170,7 +170,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -379,10 +379,8 @@
     <col min="16" max="16" width="14" customWidth="1"/>
     <col min="17" max="17" width="14" customWidth="1"/>
     <col min="18" max="18" width="14" customWidth="1"/>
-    <col min="19" max="19" width="14" customWidth="1"/>
+    <col min="19" max="19" width="58" customWidth="1"/>
     <col min="20" max="20" width="14" customWidth="1"/>
-    <col min="21" max="21" width="58" customWidth="1"/>
-    <col min="22" max="22" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -458,40 +456,30 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>F16; output mask: U32</t>
+          <t>FP8/FP4/e8m0; exact pair depends on RoundMode/SaturationMode</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>FP8/FP4/e8m0; exact pair depends on RoundMode/SaturationMode</t>
+          <t>Input: S32</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Input: S32</t>
+          <t>Input: U32</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Input: U32</t>
+          <t>U8/S8/U16/S16/U32/S32/F16/BF16/F32; NORM row-major; 4x32/4x16/4x8; scalar broadcast</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>S16; output mask: U32</t>
+          <t>Evidence / Notes</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>U8/S8/U16/S16/U32/S32/F16/BF16/F32; NORM row-major; 4x32/4x16/4x8; scalar broadcast</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Evidence / Notes</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Last checked</t>
         </is>
@@ -588,25 +576,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S2" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T2" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U2" s="7" t="inlineStr">
+      <c r="S2" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_unary_profiles
 Automated current-ISA profile verification; evidence refs: tabs_f16.</t>
         </is>
       </c>
-      <c r="V2" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T2" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -701,25 +679,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S3" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T3" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U3" s="7" t="inlineStr">
+      <c r="S3" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_basic_byte_float_profiles; v058_tepl_basic_integer_profiles
 Automated current-ISA profile verification; evidence refs: tadd_u16.</t>
         </is>
       </c>
-      <c r="V3" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T3" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -814,25 +782,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S4" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T4" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U4" s="7" t="inlineStr">
+      <c r="S4" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_scalar_arithmetic_byte_float_profiles; v058_tepl_scalar_arithmetic_integer_profiles
 Automated current-ISA profile verification; evidence refs: tadds_u16.</t>
         </is>
       </c>
-      <c r="V4" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T4" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -927,25 +885,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S5" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T5" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U5" s="7" t="inlineStr">
+      <c r="S5" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_logical_byte_profiles; v058_tepl_logical_word_half_profiles
 Automated current-ISA profile verification; evidence refs: tand_u16.</t>
         </is>
       </c>
-      <c r="V5" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T5" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -1040,25 +988,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S6" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T6" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U6" s="7" t="inlineStr">
+      <c r="S6" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_scalar_logical_byte_profiles; v058_tepl_scalar_logical_word_half_profiles
 Automated current-ISA profile verification; evidence refs: tands_u16.</t>
         </is>
       </c>
-      <c r="V6" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T6" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -1108,9 +1046,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
@@ -1133,9 +1071,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O7" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="O7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="P7" s="6" t="inlineStr">
@@ -1143,35 +1081,25 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q7" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="R7" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="S7" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T7" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U7" s="7" t="inlineStr">
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S7" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_compare_byte_float_profiles; v058_tepl_compare_integer_profiles
 Automated current-ISA profile verification; evidence refs: tcmp_u16_gt.</t>
         </is>
       </c>
-      <c r="V7" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T7" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -1201,9 +1129,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -1251,14 +1179,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="P8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Q8" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="R8" s="6" t="inlineStr">
@@ -1266,25 +1194,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S8" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U8" s="7" t="inlineStr">
+      <c r="S8" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_compare_scalar_modes; v058_tepl_compare_scalar_profiles
 Automated current-ISA profile verification; evidence refs: tcmps_u16_gt.</t>
         </is>
       </c>
-      <c r="V8" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T8" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -1359,14 +1277,14 @@
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="O9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="P9" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="P9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="Q9" s="6" t="inlineStr">
@@ -1379,22 +1297,12 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U9" s="7" t="inlineStr">
+      <c r="S9" s="7" t="inlineStr">
         <is>
           <t>QEMU TCVT now accepts B.DATR PadValue (Zero/Max/Min/Null) per B.DATR.md PadValue table; the previous TEPL DATR gate rejected PadValue on TCVT. 91-case rerun: tmov/tcvt/cast_back*/expand_to_mhc_bwd/fused_weight/reduce_fused/swiglu PASS. Cell stays UNVERIFIED because bin ELFs are regression material, not independent numeric golden.</t>
         </is>
       </c>
-      <c r="V9" s="7" t="inlineStr">
+      <c r="T9" s="7" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
@@ -1491,22 +1399,12 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S10" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T10" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U10" s="7" t="inlineStr">
+      <c r="S10" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="V10" s="7" t="inlineStr">
+      <c r="T10" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1603,25 +1501,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U11" s="7" t="inlineStr">
+      <c r="S11" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_scalar_div_profiles
 Automated current-ISA profile verification; evidence refs: tdivs_f16.</t>
         </is>
       </c>
-      <c r="V11" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T11" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -1711,30 +1599,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="R12" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="S12" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T12" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="U12" s="7" t="inlineStr">
+      <c r="R12" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="S12" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_expands_profiles
 Automated current-ISA profile verification; evidence refs: texpands_u8, texpands_s8, texpands_u16, texpands_s16, texpands_u32, texpands_s32, texpands_f16, texpands_bf16, texpands_f32.</t>
         </is>
       </c>
-      <c r="V12" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T12" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -1829,25 +1707,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S13" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T13" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U13" s="7" t="inlineStr">
+      <c r="S13" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_tfma_f32
 Automated current-ISA profile verification; evidence refs: tfma_f32.</t>
         </is>
       </c>
-      <c r="V13" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T13" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -1942,25 +1810,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S14" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T14" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U14" s="7" t="inlineStr">
+      <c r="S14" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_basic_byte_float_profiles; v058_tepl_basic_integer_profiles
 Automated current-ISA profile verification; evidence refs: tmax_u16.</t>
         </is>
       </c>
-      <c r="V14" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T14" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -2055,25 +1913,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S15" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T15" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U15" s="7" t="inlineStr">
+      <c r="S15" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_scalar_minmax_float_profiles; v058_tepl_scalar_minmax_integer_profiles
 Automated current-ISA profile verification; evidence refs: tmaxs_u8.</t>
         </is>
       </c>
-      <c r="V15" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T15" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -2168,25 +2016,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S16" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T16" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U16" s="7" t="inlineStr">
+      <c r="S16" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_basic_byte_float_profiles; v058_tepl_basic_integer_profiles
 Automated current-ISA profile verification; evidence refs: tmin_u16.</t>
         </is>
       </c>
-      <c r="V16" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T16" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -2281,25 +2119,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S17" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T17" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U17" s="7" t="inlineStr">
+      <c r="S17" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_scalar_minmax_float_profiles; v058_tepl_scalar_minmax_integer_profiles
 Automated current-ISA profile verification; evidence refs: tmins_u8.</t>
         </is>
       </c>
-      <c r="V17" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T17" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -2394,25 +2222,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S18" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T18" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U18" s="7" t="inlineStr">
+      <c r="S18" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_sub_mul_byte_float_profiles; v058_tepl_sub_mul_integer_profiles
 Automated current-ISA profile verification; evidence refs: tmul_u16.</t>
         </is>
       </c>
-      <c r="V18" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T18" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -2507,25 +2325,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S19" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T19" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U19" s="7" t="inlineStr">
+      <c r="S19" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_scalar_arithmetic_byte_float_profiles; v058_tepl_scalar_arithmetic_integer_profiles
 Automated current-ISA profile verification; evidence refs: tmuls_u16.</t>
         </is>
       </c>
-      <c r="V19" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T19" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -2620,25 +2428,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S20" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T20" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U20" s="7" t="inlineStr">
+      <c r="S20" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_unary_profiles
 Automated current-ISA profile verification; evidence refs: tneg_bf16.</t>
         </is>
       </c>
-      <c r="V20" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T20" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -2733,25 +2531,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S21" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T21" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U21" s="7" t="inlineStr">
+      <c r="S21" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_logical_byte_profiles; v058_tepl_logical_word_half_profiles
 Automated current-ISA profile verification; evidence refs: tnot_u16.</t>
         </is>
       </c>
-      <c r="V21" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T21" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -2846,25 +2634,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S22" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T22" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U22" s="7" t="inlineStr">
+      <c r="S22" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_logical_byte_profiles; v058_tepl_logical_word_half_profiles
 Automated current-ISA profile verification; evidence refs: tor_u16.</t>
         </is>
       </c>
-      <c r="V22" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T22" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -2959,25 +2737,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U23" s="7" t="inlineStr">
+      <c r="S23" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_scalar_logical_byte_profiles; v058_tepl_scalar_logical_word_half_profiles
 Automated current-ISA profile verification; evidence refs: tors_u16.</t>
         </is>
       </c>
-      <c r="V23" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T23" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -3072,25 +2840,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S24" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T24" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U24" s="7" t="inlineStr">
+      <c r="S24" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_unary_profiles
 Automated current-ISA profile verification; evidence refs: trelu_s32.</t>
         </is>
       </c>
-      <c r="V24" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T24" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -3185,22 +2943,12 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U25" s="7" t="inlineStr">
+      <c r="S25" s="7" t="inlineStr">
         <is>
           <t>Zero divisors are data content, not an encoding/descriptor legality condition (TREM.md defines only element-wise remainder with divisor-signed remainder). QEMU no longer rejects divisor tiles containing 0; QEMU returns 0 for zero divisor while gfrun returns all-1s. ISA does not define the zero-divisor value, so the cell stays UNVERIFIED.</t>
         </is>
       </c>
-      <c r="V25" s="7" t="inlineStr">
+      <c r="T25" s="7" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
@@ -3297,22 +3045,12 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S26" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T26" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U26" s="7" t="inlineStr">
+      <c r="S26" s="7" t="inlineStr">
         <is>
           <t>Zero divisors are data content, not an encoding/descriptor legality condition (TREMS.md defines only element-wise remainder). QEMU no longer rejects divisor tiles containing 0; QEMU returns 0 for zero divisor while gfrun returns all-1s. ISA does not define the zero-divisor value, so the cell stays UNVERIFIED.</t>
         </is>
       </c>
-      <c r="V26" s="7" t="inlineStr">
+      <c r="T26" s="7" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
@@ -3409,25 +3147,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S27" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T27" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U27" s="7" t="inlineStr">
+      <c r="S27" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_select_byte_profiles; v058_tepl_select_word_half_profiles
 Automated current-ISA profile verification; evidence refs: tsel_s16.</t>
         </is>
       </c>
-      <c r="V27" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T27" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -3522,25 +3250,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S28" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T28" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U28" s="7" t="inlineStr">
+      <c r="S28" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_select_byte_profiles; v058_tepl_select_word_half_profiles
 Automated current-ISA profile verification; evidence refs: tsels_u16.</t>
         </is>
       </c>
-      <c r="V28" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T28" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -3635,25 +3353,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S29" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T29" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U29" s="7" t="inlineStr">
+      <c r="S29" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_shift_profiles
 Automated current-ISA profile verification; evidence refs: tshl_u8.</t>
         </is>
       </c>
-      <c r="V29" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T29" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -3748,25 +3456,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S30" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T30" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U30" s="7" t="inlineStr">
+      <c r="S30" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_scalar_shift_profiles
 Automated current-ISA profile verification; evidence refs: tshls_u8.</t>
         </is>
       </c>
-      <c r="V30" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T30" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -3861,25 +3559,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S31" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T31" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U31" s="7" t="inlineStr">
+      <c r="S31" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_shift_profiles
 Automated current-ISA profile verification; evidence refs: tshr_u8.</t>
         </is>
       </c>
-      <c r="V31" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T31" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -3974,25 +3662,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S32" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T32" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U32" s="7" t="inlineStr">
+      <c r="S32" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_scalar_shift_profiles
 Automated current-ISA profile verification; evidence refs: tshrs_u8.</t>
         </is>
       </c>
-      <c r="V32" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T32" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -4087,25 +3765,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S33" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T33" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U33" s="7" t="inlineStr">
+      <c r="S33" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_sub_mul_byte_float_profiles; v058_tepl_sub_mul_integer_profiles
 Automated current-ISA profile verification; evidence refs: tsub_u16.</t>
         </is>
       </c>
-      <c r="V33" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T33" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -4200,25 +3868,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S34" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T34" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U34" s="7" t="inlineStr">
+      <c r="S34" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_scalar_arithmetic_byte_float_profiles; v058_tepl_scalar_arithmetic_integer_profiles
 Automated current-ISA profile verification; evidence refs: tsubs_s16.</t>
         </is>
       </c>
-      <c r="V34" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T34" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -4313,25 +3971,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S35" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T35" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U35" s="7" t="inlineStr">
+      <c r="S35" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_logical_byte_profiles; v058_tepl_logical_word_half_profiles
 Automated current-ISA profile verification; evidence refs: txor_u16.</t>
         </is>
       </c>
-      <c r="V35" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T35" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -4426,30 +4074,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S36" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T36" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U36" s="7" t="inlineStr">
+      <c r="S36" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_scalar_logical_byte_profiles; v058_tepl_scalar_logical_word_half_profiles
 Automated current-ISA profile verification; evidence refs: txors_u16.</t>
         </is>
       </c>
-      <c r="V36" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
+      <c r="T36" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V36"/>
+  <autoFilter ref="A1:T36"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>
@@ -4879,7 +4517,7 @@
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -5456,7 +5094,7 @@
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -6993,7 +6631,7 @@
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -7186,7 +6824,7 @@
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -7379,7 +7017,7 @@
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -7572,7 +7210,7 @@
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -8341,7 +7979,7 @@
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -8918,7 +8556,7 @@
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -11419,7 +11057,7 @@
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -12956,7 +12594,7 @@
       </c>
       <c r="AL44" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -13149,7 +12787,7 @@
       </c>
       <c r="AL45" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -13342,7 +12980,7 @@
       </c>
       <c r="AL46" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -13535,7 +13173,7 @@
       </c>
       <c r="AL47" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -14688,7 +14326,7 @@
       </c>
       <c r="AL53" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -15316,7 +14954,7 @@
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -16272,12 +15910,12 @@
       <c r="AK8" s="7" t="inlineStr">
         <is>
           <t>v058_tload_fp16_tile_state; v058_tload_tile_state; v058_tload_tstore_common_profiles
-Automated current-ISA profile verification; evidence refs: T#1.</t>
+Automated current-ISA profile verification; evidence refs: fp32_row0, fp32_row1, s16_row0, s16_row1, s8_row0, s8_row1, u8_row0, u8_row1, u16_row0, u16_row1, s32_row0, s32_row1, u32_row0, u32_row1, zero_stride_rows.</t>
         </is>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -16855,7 +16493,7 @@
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -17070,7 +16708,7 @@
       </c>
       <c r="R2" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -17163,7 +16801,7 @@
       </c>
       <c r="R3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -17256,7 +16894,7 @@
       </c>
       <c r="R4" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -17349,7 +16987,7 @@
       </c>
       <c r="R5" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -17442,7 +17080,7 @@
       </c>
       <c r="R6" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -17535,7 +17173,7 @@
       </c>
       <c r="R7" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -17628,7 +17266,7 @@
       </c>
       <c r="R8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -17721,7 +17359,7 @@
       </c>
       <c r="R9" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -17814,7 +17452,7 @@
       </c>
       <c r="R10" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -17907,7 +17545,7 @@
       </c>
       <c r="R11" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -18000,7 +17638,7 @@
       </c>
       <c r="R12" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -18093,7 +17731,7 @@
       </c>
       <c r="R13" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tile): update shared-ab profile status
</commit_message>
<xml_diff>
--- a/docs/linxisa/qemu_tile_profile_support.xlsx
+++ b/docs/linxisa/qemu_tile_profile_support.xlsx
@@ -170,7 +170,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -310,10 +310,10 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C11" s="3">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D11" s="4">
         <v>12</v>
@@ -323,7 +323,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>52.0%</t>
         </is>
       </c>
     </row>
@@ -334,10 +334,10 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="C12" s="3">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D12" s="4">
         <v>280</v>
@@ -347,7 +347,7 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>43.4%</t>
+          <t>43.5%</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="T2" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
       </c>
       <c r="T3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -790,7 +790,7 @@
       </c>
       <c r="T4" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
       </c>
       <c r="T5" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="T6" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="T7" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -1202,7 +1202,7 @@
       </c>
       <c r="T8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -1509,7 +1509,7 @@
       </c>
       <c r="T11" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="T12" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="T13" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -1818,7 +1818,7 @@
       </c>
       <c r="T14" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -1921,7 +1921,7 @@
       </c>
       <c r="T15" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -2024,7 +2024,7 @@
       </c>
       <c r="T16" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="T17" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -2230,7 +2230,7 @@
       </c>
       <c r="T18" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -2333,7 +2333,7 @@
       </c>
       <c r="T19" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="T20" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -2539,7 +2539,7 @@
       </c>
       <c r="T21" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -2642,7 +2642,7 @@
       </c>
       <c r="T22" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -2745,7 +2745,7 @@
       </c>
       <c r="T23" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -2848,7 +2848,7 @@
       </c>
       <c r="T24" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -3155,7 +3155,7 @@
       </c>
       <c r="T27" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -3258,7 +3258,7 @@
       </c>
       <c r="T28" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -3361,7 +3361,7 @@
       </c>
       <c r="T29" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -3464,7 +3464,7 @@
       </c>
       <c r="T30" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -3567,7 +3567,7 @@
       </c>
       <c r="T31" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -3670,7 +3670,7 @@
       </c>
       <c r="T32" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -3773,7 +3773,7 @@
       </c>
       <c r="T33" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -3876,7 +3876,7 @@
       </c>
       <c r="T34" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -3979,7 +3979,7 @@
       </c>
       <c r="T35" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -4082,7 +4082,7 @@
       </c>
       <c r="T36" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -4517,7 +4517,7 @@
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -5094,7 +5094,7 @@
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -6631,7 +6631,7 @@
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -6824,7 +6824,7 @@
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -7017,7 +7017,7 @@
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -7210,7 +7210,7 @@
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -7979,7 +7979,7 @@
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -8556,7 +8556,7 @@
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -11057,7 +11057,7 @@
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -12594,7 +12594,7 @@
       </c>
       <c r="AL44" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -12787,7 +12787,7 @@
       </c>
       <c r="AL45" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -12980,7 +12980,7 @@
       </c>
       <c r="AL46" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -13173,7 +13173,7 @@
       </c>
       <c r="AL47" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -14326,7 +14326,7 @@
       </c>
       <c r="AL53" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -14954,7 +14954,7 @@
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -15915,7 +15915,7 @@
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -16493,7 +16493,7 @@
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -16523,8 +16523,9 @@
     <col min="14" max="14" width="14" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
     <col min="16" max="16" width="14" customWidth="1"/>
-    <col min="17" max="17" width="58" customWidth="1"/>
-    <col min="18" max="18" width="14" customWidth="1"/>
+    <col min="17" max="17" width="14" customWidth="1"/>
+    <col min="18" max="18" width="58" customWidth="1"/>
+    <col min="19" max="19" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16610,10 +16611,15 @@
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
+          <t>Shared Left F32xF32 + Shared Right F32xF32 -&gt; Local F32 D; NORM; Core4; M=N=K=32; 4KB per PE</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
           <t>Evidence / Notes</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Last checked</t>
         </is>
@@ -16700,15 +16706,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q2" s="7" t="inlineStr">
+      <c r="Q2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R2" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tgemv_s32
 Automated current-ISA profile verification; evidence refs: single_tgemv_s32_m4_k4_col8.</t>
         </is>
       </c>
-      <c r="R2" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
+      <c r="S2" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -16793,15 +16804,20 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="Q3" s="7" t="inlineStr">
+      <c r="Q3" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R3" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tgemv_acc_s32
 Automated current-ISA profile verification; evidence refs: single_tgemv_acc_s32_m4_k4_explicit_c.</t>
         </is>
       </c>
-      <c r="R3" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
+      <c r="S3" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -16886,15 +16902,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q4" s="7" t="inlineStr">
+      <c r="Q4" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R4" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tgemv_bias_s32
 Automated current-ISA profile verification; evidence refs: single_tgemv_bias_s32_m4_k4_scalar_bias.</t>
         </is>
       </c>
-      <c r="R4" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
+      <c r="S4" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -16979,15 +17000,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q5" s="7" t="inlineStr">
+      <c r="Q5" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R5" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tgemv_mx_e4m3
 Automated current-ISA profile verification; evidence refs: single_tgemv_mx_e4m3_m4_k4.</t>
         </is>
       </c>
-      <c r="R5" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
+      <c r="S5" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -17072,15 +17098,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q6" s="7" t="inlineStr">
+      <c r="Q6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R6" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tgemv_mx_acc_e4m3
 Automated current-ISA profile verification; evidence refs: single_tgemv_mx_acc_e4m3_explicit_c.</t>
         </is>
       </c>
-      <c r="R6" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
+      <c r="S6" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -17165,15 +17196,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q7" s="7" t="inlineStr">
+      <c r="Q7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R7" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tgemv_mx_bias_e4m3
 Automated current-ISA profile verification; evidence refs: single_tgemv_mx_bias_e4m3_scalar_bias.</t>
         </is>
       </c>
-      <c r="R7" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
+      <c r="S7" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -17258,15 +17294,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q8" s="7" t="inlineStr">
-        <is>
-          <t>v058_cube_tmatmul_s32
-Automated current-ISA profile verification; evidence refs: single_tmatmul_s32_m4_n8_k4_col8.</t>
+      <c r="Q8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>v058_cube_tmatmul_s32; v058_cube_tmatmul_shared_ab_fp32
+Automated current-ISA profile verification; evidence refs: shared_ab_tmatmul_fp32_m32_n32_k32.</t>
+        </is>
+      </c>
+      <c r="S8" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -17351,15 +17392,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q9" s="7" t="inlineStr">
+      <c r="Q9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R9" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tmatmul_acc_s32
 Automated current-ISA profile verification; evidence refs: single_tmatmul_acc_s32_m4_n8_k4_explicit_c.</t>
         </is>
       </c>
-      <c r="R9" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
+      <c r="S9" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -17444,15 +17490,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q10" s="7" t="inlineStr">
+      <c r="Q10" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R10" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tmatmul_bias_s32
 Automated current-ISA profile verification; evidence refs: single_tmatmul_bias_s32_m4_n8_k4_row_bias.</t>
         </is>
       </c>
-      <c r="R10" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
+      <c r="S10" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -17537,15 +17588,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q11" s="7" t="inlineStr">
+      <c r="Q11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R11" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tmatmul_mx_e4m3
 Automated current-ISA profile verification; evidence refs: single_tmatmul_mx_e4m3_m4_n8_k4.</t>
         </is>
       </c>
-      <c r="R11" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
+      <c r="S11" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -17630,15 +17686,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q12" s="7" t="inlineStr">
+      <c r="Q12" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R12" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tmatmul_mx_acc_e4m3
 Automated current-ISA profile verification; evidence refs: single_tmatmul_mx_acc_e4m3_explicit_c.</t>
         </is>
       </c>
-      <c r="R12" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
+      <c r="S12" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -17723,20 +17784,25 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q13" s="7" t="inlineStr">
+      <c r="Q13" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R13" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tmatmul_mx_bias_e4m3
 Automated current-ISA profile verification; evidence refs: single_tmatmul_mx_bias_e4m3_row_bias.</t>
         </is>
       </c>
-      <c r="R13" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
+      <c r="S13" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R13"/>
+  <autoFilter ref="A1:S13"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>

</xml_diff>